<commit_message>
feat: add manual vs automation comparison
</commit_message>
<xml_diff>
--- a/07-validation/CR-09_量化验证表.xlsx
+++ b/07-validation/CR-09_量化验证表.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="量化验证表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工vs自动化对比" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +30,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -42,8 +46,28 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,13 +75,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -898,4 +954,320 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>本表基于项目实际运行记录和团队经验估算，用于评估舱路雷达对人工流程的替代价值；时间口径为单次周度情报生成。</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr"/>
+      <c r="D1" s="2" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>对比维度</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>人工操作</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>舱路雷达自动化</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>提升</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>数据收集时间</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>60-90分钟（查5个网站）</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>5分钟（读取CSV）</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>12-18倍</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>计算分析时间</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>45-60分钟（Excel公式+透视表）</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>3-5分钟（自动计算）</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>12-15倍</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>报告撰写时间</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>60-90分钟（整理文字+做PPT）</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>5-10分钟（自动生成）</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>6-12倍</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>易错点</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>公式错误、汇率日期错、单位混淆（TEU/FEU）</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>公式固化、单位自动转换、日期自动对齐</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>显著降低</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>遗漏率</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>容易漏看某航线公告、漏算某周汇率</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>26周全量扫描，不遗漏</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>从“可能遗漏”到“全量覆盖”</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>经验依赖度</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>高度依赖资深运营经验判断</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>规则映射+数据驱动，降低对个人经验的依赖</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>可复制</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>复用难度</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>每周重新做一遍，无法沉淀</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>每周替换CSV复跑，历史数据自动归档</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>可持续</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>决策一致性</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>不同人判断标准不同</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>同一规则，同一输出</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>标准化</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>证据索引</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>03-analysis/CR-04A_指标计算结果.xlsx</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>指标计算与质量等级标注</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>证据索引</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>04-decision-report/CR-04B_业务决策建议.md</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>差异化业务建议与成本场景建议</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>证据索引</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>04-decision-report/CR-05_分析报告.md</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>周度分析报告与数据质量限制</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>证据索引</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>03-analysis/rerun-simulations/week2-prime/；03-analysis/rerun-simulations/week3-prime/</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>模拟复跑验证输入不同、输出不同</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>